<commit_message>
when looking for consecutives ignore missing columns
</commit_message>
<xml_diff>
--- a/tests/testthat/testdata/examples.xlsx
+++ b/tests/testthat/testdata/examples.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding_repos\tidysheet\tests\testthat\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A819241-8965-45A6-A1A5-EB8CE3600937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4ED747-A400-4AF7-863A-D894C9A4A037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4428" yWindow="6876" windowWidth="20688" windowHeight="9960" firstSheet="1" activeTab="3" xr2:uid="{8B619997-7315-4B37-8480-7612D0E19413}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{8B619997-7315-4B37-8480-7612D0E19413}"/>
   </bookViews>
   <sheets>
     <sheet name="demo" sheetId="11" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="207">
   <si>
     <t>Example 1 2023-24</t>
   </si>
@@ -937,7 +937,7 @@
     <xf numFmtId="9" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyAlignment="1">
@@ -1037,6 +1037,13 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1048,14 +1055,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -1438,14 +1437,14 @@
   <dimension ref="A1:R21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.6328125" customWidth="1"/>
-    <col min="2" max="2" width="12.36328125" customWidth="1"/>
-    <col min="12" max="12" width="14.08984375" customWidth="1"/>
-    <col min="13" max="13" width="12.6328125" customWidth="1"/>
-    <col min="17" max="17" width="14.1796875" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" customWidth="1"/>
+    <col min="12" max="12" width="14.109375" customWidth="1"/>
+    <col min="13" max="13" width="12.6640625" customWidth="1"/>
+    <col min="17" max="17" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="21">
+    <row r="1" spans="1:18" ht="20.25">
       <c r="A1" s="12" t="s">
         <v>168</v>
       </c>
@@ -1477,19 +1476,19 @@
     </row>
     <row r="5" spans="1:18">
       <c r="B5" s="1"/>
-      <c r="C5" s="47" t="s">
+      <c r="C5" s="50" t="s">
         <v>165</v>
       </c>
-      <c r="D5" s="47"/>
-      <c r="E5" s="46" t="s">
+      <c r="D5" s="50"/>
+      <c r="E5" s="49" t="s">
         <v>166</v>
       </c>
-      <c r="F5" s="46"/>
+      <c r="F5" s="49"/>
       <c r="R5" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.6">
+    <row r="6" spans="1:18" ht="15.75">
       <c r="B6" s="13"/>
       <c r="C6" s="14" t="s">
         <v>18</v>
@@ -1657,12 +1656,12 @@
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="19.54296875" customWidth="1"/>
+    <col min="3" max="3" width="19.5546875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="11" max="11" width="11.453125" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.399999999999999">
+    <row r="1" spans="1:6" ht="18">
       <c r="A1" s="34" t="s">
         <v>82</v>
       </c>
@@ -1693,12 +1692,12 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="C8" s="49" t="s">
+      <c r="C8" s="52" t="s">
         <v>147</v>
       </c>
-      <c r="D8" s="49"/>
-      <c r="E8" s="49"/>
-      <c r="F8" s="49"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
     </row>
     <row r="9" spans="1:6">
       <c r="C9" t="s">
@@ -2007,10 +2006,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.54296875" customWidth="1"/>
+    <col min="1" max="1" width="22.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17.399999999999999">
+    <row r="1" spans="1:4" ht="18">
       <c r="A1" s="34" t="s">
         <v>131</v>
       </c>
@@ -2093,13 +2092,13 @@
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="12.81640625" customWidth="1"/>
-    <col min="3" max="3" width="16.81640625" customWidth="1"/>
+    <col min="2" max="2" width="12.77734375" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.399999999999999">
+    <row r="1" spans="1:5" ht="18">
       <c r="A1" s="34" t="s">
         <v>163</v>
       </c>
@@ -2119,7 +2118,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.6">
+    <row r="6" spans="1:5" ht="15.75">
       <c r="C6" s="24" t="s">
         <v>145</v>
       </c>
@@ -2127,7 +2126,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.6">
+    <row r="7" spans="1:5" ht="15.75">
       <c r="A7" s="24" t="s">
         <v>140</v>
       </c>
@@ -2638,14 +2637,14 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.90625" customWidth="1"/>
-    <col min="2" max="2" width="23.36328125" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" customWidth="1"/>
-    <col min="4" max="4" width="21.6328125" customWidth="1"/>
-    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="1" max="1" width="39.88671875" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21">
+    <row r="1" spans="1:6" ht="20.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2705,7 +2704,7 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:6" ht="31.2">
+    <row r="9" spans="1:6" ht="31.5">
       <c r="A9" s="4" t="s">
         <v>1</v>
       </c>
@@ -2713,7 +2712,7 @@
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:6" ht="46.8">
+    <row r="10" spans="1:6" ht="47.25">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
@@ -2813,7 +2812,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.6">
+    <row r="15" spans="1:6" ht="15.75">
       <c r="A15" s="9" t="s">
         <v>9</v>
       </c>
@@ -2834,7 +2833,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.6">
+    <row r="16" spans="1:6" ht="15.75">
       <c r="A16" s="9"/>
       <c r="B16" s="11" t="s">
         <v>11</v>
@@ -2853,76 +2852,87 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85FC1698-D933-4548-B9C9-07E812EFABD7}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.6">
+    <row r="3" spans="1:8" ht="15.75">
       <c r="A3" s="24" t="s">
         <v>203</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="46" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="51" t="s">
+      <c r="D3" s="24" t="s">
         <v>204</v>
       </c>
       <c r="E3" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="24"/>
+      <c r="G3" s="24" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="H3" s="24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>139</v>
       </c>
-      <c r="B4" s="52">
+      <c r="B4" s="47">
         <v>10</v>
       </c>
-      <c r="C4" s="52">
+      <c r="C4" s="47">
         <v>2023</v>
       </c>
-      <c r="D4" s="53" t="s">
+      <c r="D4" s="48" t="s">
         <v>206</v>
       </c>
       <c r="E4">
         <v>20</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>139</v>
       </c>
-      <c r="B5" s="52">
+      <c r="B5" s="47">
         <v>11</v>
       </c>
-      <c r="C5" s="52">
+      <c r="C5" s="47">
         <v>2023</v>
       </c>
-      <c r="D5" s="53" t="s">
+      <c r="D5" s="48" t="s">
         <v>206</v>
       </c>
       <c r="E5">
         <v>22</v>
       </c>
-      <c r="F5">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.6">
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
     </row>
   </sheetData>
   <phoneticPr fontId="23" type="noConversion"/>
@@ -2936,11 +2946,11 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" customWidth="1"/>
-    <col min="6" max="7" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" customWidth="1"/>
+    <col min="6" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21">
+    <row r="1" spans="1:7" ht="20.25">
       <c r="A1" s="12" t="s">
         <v>151</v>
       </c>
@@ -2983,7 +2993,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.6">
+    <row r="7" spans="1:7" ht="15.75">
       <c r="A7" s="13" t="s">
         <v>149</v>
       </c>
@@ -3133,14 +3143,14 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="12.6328125" customWidth="1"/>
-    <col min="3" max="3" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="12.08984375" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" customWidth="1"/>
+    <col min="7" max="7" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21">
+    <row r="1" spans="1:8" ht="20.25">
       <c r="A1" s="12" t="s">
         <v>35</v>
       </c>
@@ -3170,7 +3180,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.6">
+    <row r="8" spans="1:8" ht="15.75">
       <c r="B8" s="24" t="s">
         <v>36</v>
       </c>
@@ -3206,7 +3216,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.6">
+    <row r="11" spans="1:8" ht="15.75">
       <c r="B11" s="20" t="s">
         <v>202</v>
       </c>
@@ -3223,12 +3233,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.6">
+    <row r="12" spans="1:8" ht="15.75">
       <c r="F12" s="24" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15.6">
+    <row r="16" spans="1:8" ht="15.75">
       <c r="B16" s="24" t="s">
         <v>38</v>
       </c>
@@ -3277,14 +3287,14 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" customWidth="1"/>
-    <col min="4" max="4" width="13.6328125" customWidth="1"/>
+    <col min="2" max="2" width="11.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
     <col min="5" max="5" width="4" customWidth="1"/>
-    <col min="6" max="6" width="14.90625" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21">
+    <row r="1" spans="1:7" ht="20.25">
       <c r="A1" s="2" t="s">
         <v>155</v>
       </c>
@@ -3323,17 +3333,17 @@
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="48" t="s">
+      <c r="B8" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="48"/>
-      <c r="D8" s="48"/>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
       <c r="E8" s="25"/>
       <c r="F8" s="26" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.6">
+    <row r="9" spans="1:7" ht="15.75">
       <c r="A9" s="31" t="s">
         <v>56</v>
       </c>
@@ -3349,7 +3359,7 @@
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="1:7" ht="15.6">
+    <row r="10" spans="1:7" ht="15.75">
       <c r="A10" s="5"/>
       <c r="B10" s="28" t="s">
         <v>49</v>
@@ -3491,15 +3501,15 @@
   <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="29.6328125" customWidth="1"/>
-    <col min="2" max="2" width="27.6328125" customWidth="1"/>
-    <col min="3" max="3" width="25.08984375" customWidth="1"/>
-    <col min="4" max="4" width="23.81640625" customWidth="1"/>
-    <col min="5" max="5" width="22.36328125" customWidth="1"/>
-    <col min="6" max="6" width="25.54296875" customWidth="1"/>
+    <col min="1" max="1" width="29.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.109375" customWidth="1"/>
+    <col min="4" max="4" width="23.77734375" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" customWidth="1"/>
+    <col min="6" max="6" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17.399999999999999">
+    <row r="1" spans="1:14" ht="18">
       <c r="A1" s="34" t="s">
         <v>107</v>
       </c>
@@ -3516,7 +3526,7 @@
       <c r="L1" s="32"/>
       <c r="M1" s="32"/>
     </row>
-    <row r="2" spans="1:14" ht="15.6">
+    <row r="2" spans="1:14" ht="15.75">
       <c r="A2" s="35" t="s">
         <v>59</v>
       </c>
@@ -3533,7 +3543,7 @@
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
     </row>
-    <row r="3" spans="1:14" ht="15.6">
+    <row r="3" spans="1:14" ht="15.75">
       <c r="A3" s="35" t="s">
         <v>60</v>
       </c>
@@ -3550,7 +3560,7 @@
       <c r="L3" s="32"/>
       <c r="M3" s="32"/>
     </row>
-    <row r="4" spans="1:14" ht="15.6">
+    <row r="4" spans="1:14" ht="15.75">
       <c r="A4" t="s">
         <v>114</v>
       </c>
@@ -3561,7 +3571,7 @@
       <c r="L4" s="32"/>
       <c r="M4" s="32"/>
     </row>
-    <row r="5" spans="1:14" s="24" customFormat="1" ht="31.2">
+    <row r="5" spans="1:14" s="24" customFormat="1" ht="31.5">
       <c r="A5" s="24" t="s">
         <v>10</v>
       </c>
@@ -3702,10 +3712,10 @@
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.1796875" customWidth="1"/>
+    <col min="1" max="1" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17.399999999999999">
+    <row r="1" spans="1:3" ht="18">
       <c r="A1" s="34" t="s">
         <v>70</v>
       </c>
@@ -3715,12 +3725,12 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="20.399999999999999" customHeight="1">
+    <row r="3" spans="1:3" ht="20.45" customHeight="1">
       <c r="A3" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="19.8" thickBot="1">
+    <row r="5" spans="1:3" ht="20.25" thickBot="1">
       <c r="A5" s="42" t="s">
         <v>156</v>
       </c>
@@ -3733,7 +3743,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.6">
+    <row r="7" spans="1:3" ht="15.75">
       <c r="A7" s="24" t="s">
         <v>10</v>
       </c>
@@ -3782,7 +3792,7 @@
       </c>
       <c r="C12" s="39"/>
     </row>
-    <row r="13" spans="1:3" ht="15.6">
+    <row r="13" spans="1:3" ht="15.75">
       <c r="A13" s="24" t="s">
         <v>10</v>
       </c>
@@ -3820,12 +3830,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="19.8" thickBot="1">
+    <row r="18" spans="1:3" ht="20.25" thickBot="1">
       <c r="A18" s="42" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="16.2" thickTop="1">
+    <row r="19" spans="1:3" ht="16.5" thickTop="1">
       <c r="B19" s="24" t="s">
         <v>159</v>
       </c>

</xml_diff>

<commit_message>
add tidy_sheet test for example 10 with all descriptor locations
</commit_message>
<xml_diff>
--- a/tests/testthat/testdata/examples.xlsx
+++ b/tests/testthat/testdata/examples.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding_repos\tidysheet\tests\testthat\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4ED747-A400-4AF7-863A-D894C9A4A037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A95544D-7FDC-4145-BAC8-D2839ABCD497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{8B619997-7315-4B37-8480-7612D0E19413}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="11" xr2:uid="{8B619997-7315-4B37-8480-7612D0E19413}"/>
   </bookViews>
   <sheets>
     <sheet name="demo" sheetId="11" r:id="rId1"/>
     <sheet name="demo_output" sheetId="12" r:id="rId2"/>
     <sheet name="example 1" sheetId="1" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="13" r:id="rId4"/>
-    <sheet name="example 2" sheetId="2" r:id="rId5"/>
-    <sheet name="example 3" sheetId="3" r:id="rId6"/>
-    <sheet name="example 4" sheetId="4" r:id="rId7"/>
-    <sheet name="example 5" sheetId="5" r:id="rId8"/>
-    <sheet name="example 6" sheetId="6" r:id="rId9"/>
-    <sheet name="example 7" sheetId="7" r:id="rId10"/>
-    <sheet name="example 8" sheetId="8" r:id="rId11"/>
-    <sheet name="example 9" sheetId="9" r:id="rId12"/>
+    <sheet name="example 2" sheetId="2" r:id="rId4"/>
+    <sheet name="example 3" sheetId="3" r:id="rId5"/>
+    <sheet name="example 4" sheetId="4" r:id="rId6"/>
+    <sheet name="example 5" sheetId="5" r:id="rId7"/>
+    <sheet name="example 6" sheetId="6" r:id="rId8"/>
+    <sheet name="example 7" sheetId="7" r:id="rId9"/>
+    <sheet name="example 8" sheetId="8" r:id="rId10"/>
+    <sheet name="example 9" sheetId="9" r:id="rId11"/>
+    <sheet name="example 10" sheetId="13" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="214">
   <si>
     <t>Example 1 2023-24</t>
   </si>
@@ -666,16 +666,37 @@
     <t>2021_2022</t>
   </si>
   <si>
-    <t>country</t>
-  </si>
-  <si>
-    <t>region</t>
-  </si>
-  <si>
-    <t>title - 2023-24</t>
-  </si>
-  <si>
-    <t>EA</t>
+    <t>item 1</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>1st</t>
+  </si>
+  <si>
+    <t>2nd</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>Total set 1</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Total set 2</t>
+  </si>
+  <si>
+    <t>Example 10 descriptors given in every possible location for a single table - 2023-24</t>
   </si>
 </sst>
 </file>
@@ -685,7 +706,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0&quot; &quot;"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -837,15 +858,8 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color theme="0" tint="-0.249977111117893"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -872,7 +886,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
+        <fgColor theme="7" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -937,7 +975,7 @@
     <xf numFmtId="9" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyAlignment="1">
@@ -1036,14 +1074,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1437,14 +1472,14 @@
   <dimension ref="A1:R21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" customWidth="1"/>
-    <col min="12" max="12" width="14.109375" customWidth="1"/>
-    <col min="13" max="13" width="12.6640625" customWidth="1"/>
-    <col min="17" max="17" width="14.21875" customWidth="1"/>
+    <col min="1" max="1" width="11.6328125" customWidth="1"/>
+    <col min="2" max="2" width="12.36328125" customWidth="1"/>
+    <col min="12" max="12" width="14.08984375" customWidth="1"/>
+    <col min="13" max="13" width="12.6328125" customWidth="1"/>
+    <col min="17" max="17" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="20.25">
+    <row r="1" spans="1:18" ht="21">
       <c r="A1" s="12" t="s">
         <v>168</v>
       </c>
@@ -1476,19 +1511,19 @@
     </row>
     <row r="5" spans="1:18">
       <c r="B5" s="1"/>
-      <c r="C5" s="50" t="s">
+      <c r="C5" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="D5" s="50"/>
-      <c r="E5" s="49" t="s">
+      <c r="D5" s="51"/>
+      <c r="E5" s="50" t="s">
         <v>166</v>
       </c>
-      <c r="F5" s="49"/>
+      <c r="F5" s="50"/>
       <c r="R5" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.75">
+    <row r="6" spans="1:18" ht="15.6">
       <c r="B6" s="13"/>
       <c r="C6" s="14" t="s">
         <v>18</v>
@@ -1652,526 +1687,323 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4F711F3-0143-4CD6-8E8C-CF04959145E6}">
-  <dimension ref="A1:F32"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB23A844-51C0-4B06-8B54-8E15B13CE72B}">
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="19.5546875" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="11" max="11" width="11.44140625" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18">
+    <row r="1" spans="1:4" ht="17.399999999999999">
       <c r="A1" s="34" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" customHeight="1">
       <c r="A3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" customHeight="1">
       <c r="A4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="C8" s="52" t="s">
-        <v>147</v>
-      </c>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="C9" t="s">
-        <v>160</v>
-      </c>
-      <c r="D9" t="s">
-        <v>99</v>
-      </c>
-      <c r="F9" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="C10" t="s">
-        <v>98</v>
-      </c>
-      <c r="D10" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="C11" t="s">
-        <v>100</v>
-      </c>
-      <c r="D11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="C13" t="s">
-        <v>95</v>
-      </c>
-      <c r="D13" t="s">
-        <v>96</v>
-      </c>
-      <c r="F13" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15">
-        <v>2000</v>
-      </c>
-      <c r="B15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9">
         <v>1</v>
       </c>
-      <c r="D15">
-        <v>2</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="B16" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16">
-        <v>2</v>
-      </c>
-      <c r="D16">
-        <v>2</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="B17" t="s">
-        <v>81</v>
-      </c>
-      <c r="C17">
-        <v>3</v>
-      </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="B18" t="s">
-        <v>83</v>
-      </c>
-      <c r="C18">
+      <c r="C9">
         <v>4</v>
       </c>
-      <c r="D18">
-        <v>2</v>
-      </c>
-      <c r="F18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="B19" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19">
+      <c r="D9">
         <v>5</v>
       </c>
-      <c r="D19">
-        <v>2</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="B20" t="s">
-        <v>85</v>
-      </c>
-      <c r="C20">
-        <v>6</v>
-      </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="B21" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21">
-        <v>7</v>
-      </c>
-      <c r="D21">
-        <v>2</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="B22" t="s">
-        <v>87</v>
-      </c>
-      <c r="C22">
-        <v>8</v>
-      </c>
-      <c r="D22">
-        <v>2</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="B23" t="s">
-        <v>88</v>
-      </c>
-      <c r="C23">
-        <v>9</v>
-      </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24">
-        <v>2001</v>
-      </c>
-      <c r="B24" t="s">
-        <v>92</v>
-      </c>
-      <c r="C24">
-        <v>10</v>
-      </c>
-      <c r="D24">
-        <v>2</v>
-      </c>
-      <c r="F24">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="B25" t="s">
-        <v>93</v>
-      </c>
-      <c r="C25">
-        <v>11</v>
-      </c>
-      <c r="D25">
-        <v>2</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="B26" t="s">
-        <v>94</v>
-      </c>
-      <c r="C26">
-        <v>12</v>
-      </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="C27" t="s">
-        <v>146</v>
-      </c>
-      <c r="D27" t="s">
-        <v>146</v>
-      </c>
-      <c r="F27" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="C28" t="s">
-        <v>146</v>
-      </c>
-      <c r="D28" t="s">
-        <v>146</v>
-      </c>
-      <c r="F28" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" t="s">
-        <v>89</v>
-      </c>
-      <c r="C29">
-        <f>SUM(C15:C17)</f>
-        <v>6</v>
-      </c>
-      <c r="D29">
-        <v>5</v>
-      </c>
-      <c r="F29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" t="s">
-        <v>90</v>
-      </c>
-      <c r="C30">
-        <f>SUM(C18:C20)</f>
-        <v>15</v>
-      </c>
-      <c r="D30">
-        <v>5</v>
-      </c>
-      <c r="F30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" t="s">
-        <v>162</v>
-      </c>
-      <c r="C31">
-        <f>SUM(C21:C23)</f>
-        <v>24</v>
-      </c>
-      <c r="D31">
-        <v>5</v>
-      </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" t="s">
-        <v>91</v>
-      </c>
-      <c r="C32">
-        <f>SUM(C24:C26)</f>
-        <v>33</v>
-      </c>
-      <c r="D32">
-        <v>5</v>
-      </c>
-      <c r="F32">
-        <v>100</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="C8:F8"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB23A844-51C0-4B06-8B54-8E15B13CE72B}">
-  <dimension ref="A1:D9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9644BECB-6957-489A-9399-136E9FE37B99}">
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="16.81640625" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="16.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18">
+    <row r="1" spans="1:5" ht="17.399999999999999">
       <c r="A1" s="34" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" customHeight="1">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="B6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="43" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.6">
+      <c r="C6" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.6">
+      <c r="A7" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>142</v>
       </c>
       <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
         <v>3</v>
       </c>
-      <c r="D8">
+      <c r="E8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>135</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9">
-        <v>4</v>
-      </c>
-      <c r="D9">
-        <v>5</v>
+      <c r="E9">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9644BECB-6957-489A-9399-136E9FE37B99}">
-  <dimension ref="A1:E9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85FC1698-D933-4548-B9C9-07E812EFABD7}">
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="2" max="2" width="12.77734375" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18">
-      <c r="A1" s="34" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>143</v>
+    <row r="1" spans="1:5" ht="15.6">
+      <c r="A1" s="24" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>144</v>
+      <c r="B3" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="43" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15.75">
-      <c r="C6" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="E6" s="24" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15.75">
-      <c r="A7" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>141</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>137</v>
+      <c r="A4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="46" t="s">
+        <v>204</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="47" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="48" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="48" t="s">
+        <v>208</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B8" t="s">
-        <v>142</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
-      <c r="E8">
-        <v>5</v>
+      <c r="A8" s="47" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>139</v>
+      <c r="A9" s="48" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D9">
-        <v>4</v>
-      </c>
-      <c r="E9">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="49" t="s">
+        <v>210</v>
+      </c>
+      <c r="B10">
+        <v>12</v>
+      </c>
+      <c r="C10">
+        <v>15</v>
+      </c>
+      <c r="D10">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="47" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="48" t="s">
+        <v>207</v>
+      </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12">
+        <v>11</v>
+      </c>
+      <c r="D12">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="49" t="s">
+        <v>212</v>
+      </c>
+      <c r="B13">
+        <v>10</v>
+      </c>
+      <c r="C13">
+        <v>11</v>
+      </c>
+      <c r="D13">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2637,14 +2469,14 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.88671875" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" customWidth="1"/>
-    <col min="5" max="5" width="13.21875" customWidth="1"/>
+    <col min="1" max="1" width="39.90625" customWidth="1"/>
+    <col min="2" max="2" width="23.36328125" customWidth="1"/>
+    <col min="3" max="3" width="23.81640625" customWidth="1"/>
+    <col min="4" max="4" width="21.6328125" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="20.25">
+    <row r="1" spans="1:6" ht="21">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2704,7 +2536,7 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:6" ht="31.5">
+    <row r="9" spans="1:6" ht="31.2">
       <c r="A9" s="4" t="s">
         <v>1</v>
       </c>
@@ -2712,7 +2544,7 @@
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:6" ht="47.25">
+    <row r="10" spans="1:6" ht="46.8">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
@@ -2812,7 +2644,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.75">
+    <row r="15" spans="1:6" ht="15.6">
       <c r="A15" s="9" t="s">
         <v>9</v>
       </c>
@@ -2833,7 +2665,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.75">
+    <row r="16" spans="1:6" ht="15.6">
       <c r="A16" s="9"/>
       <c r="B16" s="11" t="s">
         <v>11</v>
@@ -2851,286 +2683,339 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85FC1698-D933-4548-B9C9-07E812EFABD7}">
-  <dimension ref="A1:H6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51A5631-8A8B-4394-8AE5-5EEF34362AE4}">
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" customWidth="1"/>
+    <col min="6" max="7" width="9.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75">
-      <c r="A3" s="24" t="s">
-        <v>203</v>
-      </c>
-      <c r="B3" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="C3" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="24" t="s">
-        <v>204</v>
-      </c>
-      <c r="E3" s="24" t="s">
+    <row r="1" spans="1:7" ht="21">
+      <c r="A1" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.6">
+      <c r="A7" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="22">
+        <v>45658</v>
+      </c>
+      <c r="G7" s="22">
+        <v>45717</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24" t="s">
+      <c r="B8" s="15">
+        <v>10</v>
+      </c>
+      <c r="C8" s="15">
+        <v>11</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="15">
+        <v>10</v>
+      </c>
+      <c r="G8" s="15">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B9" s="15">
+        <v>5</v>
+      </c>
+      <c r="C9" s="15">
+        <v>5</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="F9" s="15">
+        <v>5</v>
+      </c>
+      <c r="G9" s="15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="B10" s="15">
+        <v>20</v>
+      </c>
+      <c r="C10" s="15">
+        <v>32</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="15">
+        <v>20</v>
+      </c>
+      <c r="G10" s="15">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B11" s="15">
+        <v>10</v>
+      </c>
+      <c r="C11" s="15">
+        <v>20</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" s="15">
+        <v>10</v>
+      </c>
+      <c r="G11" s="15">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B12" s="15">
+        <v>10</v>
+      </c>
+      <c r="C12" s="15">
+        <v>12</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="F12" s="15">
+        <v>10</v>
+      </c>
+      <c r="G12" s="15">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="10" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B4" s="47">
-        <v>10</v>
-      </c>
-      <c r="C4" s="47">
-        <v>2023</v>
-      </c>
-      <c r="D4" s="48" t="s">
-        <v>206</v>
-      </c>
-      <c r="E4">
-        <v>20</v>
-      </c>
-      <c r="G4">
-        <v>30</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B5" s="47">
-        <v>11</v>
-      </c>
-      <c r="C5" s="47">
-        <v>2023</v>
-      </c>
-      <c r="D5" s="48" t="s">
-        <v>206</v>
-      </c>
-      <c r="E5">
+      <c r="B13" s="15">
+        <v>56</v>
+      </c>
+      <c r="C13" s="15">
+        <v>56</v>
+      </c>
+      <c r="E13" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
+      <c r="F13" s="15">
+        <v>56</v>
+      </c>
+      <c r="G13" s="15">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51A5631-8A8B-4394-8AE5-5EEF34362AE4}">
-  <dimension ref="A1:G13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53A3D49F-26FB-4041-98FA-71B10D10213D}">
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="5" max="5" width="11.21875" customWidth="1"/>
-    <col min="6" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6328125" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" customWidth="1"/>
+    <col min="5" max="5" width="12.08984375" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" customWidth="1"/>
+    <col min="7" max="7" width="10.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="20.25">
+    <row r="1" spans="1:8" ht="21">
       <c r="A1" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.6">
+      <c r="B8" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="B9" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="B10" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="19">
+        <v>100</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="19">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15.6">
+      <c r="B11" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="C11" s="21">
+        <v>200</v>
+      </c>
+      <c r="F11" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="21">
         <v>150</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="E6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.75">
-      <c r="A7" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="22">
-        <v>45658</v>
-      </c>
-      <c r="G7" s="22">
-        <v>45717</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="10" t="s">
+      <c r="H11" s="24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15.6">
+      <c r="F12" s="24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15.6">
+      <c r="B16" s="24" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4">
+      <c r="B18" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="15">
-        <v>10</v>
-      </c>
-      <c r="C8" s="15">
-        <v>11</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="C18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="19">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4">
+      <c r="B19" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="15">
-        <v>10</v>
-      </c>
-      <c r="G8" s="15">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="B9" s="15">
-        <v>5</v>
-      </c>
-      <c r="C9" s="15">
-        <v>5</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="F9" s="15">
-        <v>5</v>
-      </c>
-      <c r="G9" s="15">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="15">
-        <v>20</v>
-      </c>
-      <c r="C10" s="15">
-        <v>32</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="15">
-        <v>20</v>
-      </c>
-      <c r="G10" s="15">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="B11" s="15">
-        <v>10</v>
-      </c>
-      <c r="C11" s="15">
-        <v>20</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="F11" s="15">
-        <v>10</v>
-      </c>
-      <c r="G11" s="15">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="B12" s="15">
-        <v>10</v>
-      </c>
-      <c r="C12" s="15">
-        <v>12</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="F12" s="15">
-        <v>10</v>
-      </c>
-      <c r="G12" s="15">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="15">
-        <v>56</v>
-      </c>
-      <c r="C13" s="15">
-        <v>56</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="F13" s="15">
-        <v>56</v>
-      </c>
-      <c r="G13" s="15">
-        <v>56</v>
+      <c r="C19" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" s="21">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -3139,162 +3024,19 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53A3D49F-26FB-4041-98FA-71B10D10213D}">
-  <dimension ref="A1:H19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" customWidth="1"/>
-    <col min="7" max="7" width="10.88671875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="20.25">
-      <c r="A1" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.75">
-      <c r="B8" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="F8" s="24" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="B9" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="B10" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="19">
-        <v>100</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="19">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15.75">
-      <c r="B11" s="20" t="s">
-        <v>202</v>
-      </c>
-      <c r="C11" s="21">
-        <v>200</v>
-      </c>
-      <c r="F11" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="21">
-        <v>150</v>
-      </c>
-      <c r="H11" s="24" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15.75">
-      <c r="F12" s="24" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="15.75">
-      <c r="B16" s="24" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4">
-      <c r="B17" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" t="s">
-        <v>40</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4">
-      <c r="B18" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D18" s="19">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4">
-      <c r="B19" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="21">
-        <v>150</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E9BF5B1-5B75-440F-BCD2-E94C185D352A}">
   <dimension ref="A1:P18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="11.21875" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.1796875" customWidth="1"/>
+    <col min="3" max="3" width="11.6328125" customWidth="1"/>
+    <col min="4" max="4" width="13.6328125" customWidth="1"/>
     <col min="5" max="5" width="4" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" customWidth="1"/>
+    <col min="6" max="6" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="20.25">
+    <row r="1" spans="1:7" ht="21">
       <c r="A1" s="2" t="s">
         <v>155</v>
       </c>
@@ -3333,17 +3075,17 @@
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="51" t="s">
+      <c r="B8" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="52"/>
       <c r="E8" s="25"/>
       <c r="F8" s="26" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.75">
+    <row r="9" spans="1:7" ht="15.6">
       <c r="A9" s="31" t="s">
         <v>56</v>
       </c>
@@ -3359,7 +3101,7 @@
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="1:7" ht="15.75">
+    <row r="10" spans="1:7" ht="15.6">
       <c r="A10" s="5"/>
       <c r="B10" s="28" t="s">
         <v>49</v>
@@ -3496,20 +3238,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEF0B59E-6DC3-4942-9160-730FC61B2EF4}">
   <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="29.6640625" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.109375" customWidth="1"/>
-    <col min="4" max="4" width="23.77734375" customWidth="1"/>
-    <col min="5" max="5" width="22.33203125" customWidth="1"/>
-    <col min="6" max="6" width="25.5546875" customWidth="1"/>
+    <col min="1" max="1" width="29.6328125" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" customWidth="1"/>
+    <col min="3" max="3" width="25.08984375" customWidth="1"/>
+    <col min="4" max="4" width="23.81640625" customWidth="1"/>
+    <col min="5" max="5" width="22.36328125" customWidth="1"/>
+    <col min="6" max="6" width="25.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18">
+    <row r="1" spans="1:14" ht="17.399999999999999">
       <c r="A1" s="34" t="s">
         <v>107</v>
       </c>
@@ -3526,7 +3268,7 @@
       <c r="L1" s="32"/>
       <c r="M1" s="32"/>
     </row>
-    <row r="2" spans="1:14" ht="15.75">
+    <row r="2" spans="1:14" ht="15.6">
       <c r="A2" s="35" t="s">
         <v>59</v>
       </c>
@@ -3543,7 +3285,7 @@
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
     </row>
-    <row r="3" spans="1:14" ht="15.75">
+    <row r="3" spans="1:14" ht="15.6">
       <c r="A3" s="35" t="s">
         <v>60</v>
       </c>
@@ -3560,7 +3302,7 @@
       <c r="L3" s="32"/>
       <c r="M3" s="32"/>
     </row>
-    <row r="4" spans="1:14" ht="15.75">
+    <row r="4" spans="1:14" ht="15.6">
       <c r="A4" t="s">
         <v>114</v>
       </c>
@@ -3571,7 +3313,7 @@
       <c r="L4" s="32"/>
       <c r="M4" s="32"/>
     </row>
-    <row r="5" spans="1:14" s="24" customFormat="1" ht="31.5">
+    <row r="5" spans="1:14" s="24" customFormat="1" ht="31.2">
       <c r="A5" s="24" t="s">
         <v>10</v>
       </c>
@@ -3707,15 +3449,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B219578-77D1-4986-A64E-11C06B3659FB}">
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.21875" customWidth="1"/>
+    <col min="1" max="1" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18">
+    <row r="1" spans="1:3" ht="17.399999999999999">
       <c r="A1" s="34" t="s">
         <v>70</v>
       </c>
@@ -3725,12 +3467,12 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="20.45" customHeight="1">
+    <row r="3" spans="1:3" ht="20.399999999999999" customHeight="1">
       <c r="A3" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="20.25" thickBot="1">
+    <row r="5" spans="1:3" ht="19.8" thickBot="1">
       <c r="A5" s="42" t="s">
         <v>156</v>
       </c>
@@ -3743,7 +3485,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75">
+    <row r="7" spans="1:3" ht="15.6">
       <c r="A7" s="24" t="s">
         <v>10</v>
       </c>
@@ -3792,7 +3534,7 @@
       </c>
       <c r="C12" s="39"/>
     </row>
-    <row r="13" spans="1:3" ht="15.75">
+    <row r="13" spans="1:3" ht="15.6">
       <c r="A13" s="24" t="s">
         <v>10</v>
       </c>
@@ -3830,12 +3572,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="20.25" thickBot="1">
+    <row r="18" spans="1:3" ht="19.8" thickBot="1">
       <c r="A18" s="42" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="16.5" thickTop="1">
+    <row r="19" spans="1:3" ht="16.2" thickTop="1">
       <c r="B19" s="24" t="s">
         <v>159</v>
       </c>
@@ -3857,4 +3599,354 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4F711F3-0143-4CD6-8E8C-CF04959145E6}">
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="19.54296875" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="11" max="11" width="11.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17.399999999999999">
+      <c r="A1" s="34" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="C8" s="53" t="s">
+        <v>147</v>
+      </c>
+      <c r="D8" s="53"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="53"/>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="C9" t="s">
+        <v>160</v>
+      </c>
+      <c r="D9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="C10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="C11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="C13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15">
+        <v>2000</v>
+      </c>
+      <c r="B15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="B16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="B17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="B18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18">
+        <v>4</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="B19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="B20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="B21" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21">
+        <v>7</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="B22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22">
+        <v>8</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="B23" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23">
+        <v>9</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24">
+        <v>2001</v>
+      </c>
+      <c r="B24" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24">
+        <v>10</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="F24">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="B25" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25">
+        <v>11</v>
+      </c>
+      <c r="D25">
+        <v>2</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="B26" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26">
+        <v>12</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="C27" t="s">
+        <v>146</v>
+      </c>
+      <c r="D27" t="s">
+        <v>146</v>
+      </c>
+      <c r="F27" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="C28" t="s">
+        <v>146</v>
+      </c>
+      <c r="D28" t="s">
+        <v>146</v>
+      </c>
+      <c r="F28" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29">
+        <f>SUM(C15:C17)</f>
+        <v>6</v>
+      </c>
+      <c r="D29">
+        <v>5</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30">
+        <f>SUM(C18:C20)</f>
+        <v>15</v>
+      </c>
+      <c r="D30">
+        <v>5</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>162</v>
+      </c>
+      <c r="C31">
+        <f>SUM(C21:C23)</f>
+        <v>24</v>
+      </c>
+      <c r="D31">
+        <v>5</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32">
+        <f>SUM(C24:C26)</f>
+        <v>33</v>
+      </c>
+      <c r="D32">
+        <v>5</v>
+      </c>
+      <c r="F32">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C8:F8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add spaces to a header in examples for tidy_sheet tests
Without the new fix, test 9 would now fail
</commit_message>
<xml_diff>
--- a/tests/testthat/testdata/examples.xlsx
+++ b/tests/testthat/testdata/examples.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding_repos\tidysheet\tests\testthat\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A95544D-7FDC-4145-BAC8-D2839ABCD497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F4AFE1-4284-42E4-AB40-D3161EECAAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="11" xr2:uid="{8B619997-7315-4B37-8480-7612D0E19413}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="10" xr2:uid="{8B619997-7315-4B37-8480-7612D0E19413}"/>
   </bookViews>
   <sheets>
     <sheet name="demo" sheetId="11" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="215">
   <si>
     <t>Example 1 2023-24</t>
   </si>
@@ -588,9 +588,6 @@
     <t>year_type</t>
   </si>
   <si>
-    <t>fy_start</t>
-  </si>
-  <si>
     <t>C6</t>
   </si>
   <si>
@@ -697,6 +694,12 @@
   </si>
   <si>
     <t>Example 10 descriptors given in every possible location for a single table - 2023-24</t>
+  </si>
+  <si>
+    <t>There are spaces in D7 - it is not a blank cell so without the refine_blanks function it would lead to column D values having a blank where other values have 'description A' (all values should get a value of 'description A')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
   </si>
 </sst>
 </file>
@@ -1469,17 +1472,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6C12350-3FC9-4A16-9BD3-0EB8F46D2BAE}">
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.6328125" customWidth="1"/>
-    <col min="2" max="2" width="12.36328125" customWidth="1"/>
-    <col min="12" max="12" width="14.08984375" customWidth="1"/>
-    <col min="13" max="13" width="12.6328125" customWidth="1"/>
-    <col min="17" max="17" width="14.1796875" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" customWidth="1"/>
+    <col min="12" max="12" width="14.109375" customWidth="1"/>
+    <col min="13" max="13" width="12.6640625" customWidth="1"/>
+    <col min="17" max="17" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="21">
+    <row r="1" spans="1:6" ht="20.25">
       <c r="A1" s="12" t="s">
         <v>168</v>
       </c>
@@ -1487,7 +1490,7 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>169</v>
       </c>
@@ -1495,21 +1498,21 @@
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:6">
       <c r="B5" s="1"/>
       <c r="C5" s="51" t="s">
         <v>165</v>
@@ -1519,11 +1522,8 @@
         <v>166</v>
       </c>
       <c r="F5" s="50"/>
-      <c r="R5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="15.6">
+    </row>
+    <row r="6" spans="1:6" ht="15.75">
       <c r="B6" s="13"/>
       <c r="C6" s="14" t="s">
         <v>18</v>
@@ -1537,11 +1537,8 @@
       <c r="F6" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="R6">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18">
+    </row>
+    <row r="7" spans="1:6">
       <c r="B7" s="10" t="s">
         <v>20</v>
       </c>
@@ -1557,11 +1554,8 @@
       <c r="F7" s="15">
         <v>13</v>
       </c>
-      <c r="R7">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18">
+    </row>
+    <row r="8" spans="1:6">
       <c r="B8" s="10" t="s">
         <v>167</v>
       </c>
@@ -1577,11 +1571,8 @@
       <c r="F8" s="15">
         <v>14</v>
       </c>
-      <c r="R8">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18">
+    </row>
+    <row r="9" spans="1:6">
       <c r="B9" s="10" t="s">
         <v>21</v>
       </c>
@@ -1597,11 +1588,8 @@
       <c r="F9" s="15">
         <v>15</v>
       </c>
-      <c r="R9">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18">
+    </row>
+    <row r="10" spans="1:6">
       <c r="B10" s="10" t="s">
         <v>167</v>
       </c>
@@ -1617,65 +1605,9 @@
       <c r="F10" s="15">
         <v>16</v>
       </c>
-      <c r="R10">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18">
-      <c r="R11">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18">
-      <c r="R12">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18">
-      <c r="R13">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18">
+    </row>
+    <row r="14" spans="1:6">
       <c r="B14" s="44"/>
-      <c r="R14">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18">
-      <c r="R15">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18">
-      <c r="R16">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="17" spans="18:18">
-      <c r="R17">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="18" spans="18:18">
-      <c r="R18">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="19" spans="18:18">
-      <c r="R19">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="20" spans="18:18">
-      <c r="R20">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="21" spans="18:18">
-      <c r="R21">
-        <v>2020</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1691,10 +1623,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.54296875" customWidth="1"/>
+    <col min="1" max="1" width="22.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17.399999999999999">
+    <row r="1" spans="1:4" ht="18">
       <c r="A1" s="34" t="s">
         <v>131</v>
       </c>
@@ -1774,16 +1706,16 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9644BECB-6957-489A-9399-136E9FE37B99}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="12.81640625" customWidth="1"/>
-    <col min="3" max="3" width="16.81640625" customWidth="1"/>
+    <col min="2" max="2" width="12.77734375" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.399999999999999">
+    <row r="1" spans="1:5" ht="18">
       <c r="A1" s="34" t="s">
         <v>163</v>
       </c>
@@ -1803,59 +1735,67 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.6">
-      <c r="C6" s="24" t="s">
+    <row r="5" spans="1:5">
+      <c r="A5" s="43" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.75">
+      <c r="C7" s="24" t="s">
         <v>145</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="D7" t="s">
+        <v>214</v>
+      </c>
+      <c r="E7" s="24" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.6">
-      <c r="A7" s="24" t="s">
+    <row r="8" spans="1:5" ht="15.75">
+      <c r="A8" s="24" t="s">
         <v>140</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B8" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C8" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D8" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E8" s="24" t="s">
         <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B8" t="s">
-        <v>142</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
-      <c r="E8">
-        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>139</v>
       </c>
+      <c r="B9" t="s">
+        <v>142</v>
+      </c>
       <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10">
         <v>2</v>
       </c>
-      <c r="D9">
+      <c r="D10">
         <v>4</v>
       </c>
-      <c r="E9">
+      <c r="E10">
         <v>6</v>
       </c>
     </row>
@@ -1870,9 +1810,9 @@
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6">
+    <row r="1" spans="1:5" ht="15.75">
       <c r="A1" s="24" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1886,7 +1826,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B4" s="46" t="s">
         <v>22</v>
@@ -1895,20 +1835,20 @@
         <v>61</v>
       </c>
       <c r="D4" s="46" t="s">
+        <v>203</v>
+      </c>
+      <c r="E4" s="18" t="s">
         <v>204</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="47" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="48" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1925,7 +1865,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="48" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B7">
         <v>4</v>
@@ -1939,12 +1879,12 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="47" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="48" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B9">
         <v>7</v>
@@ -1961,7 +1901,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="49" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B10">
         <v>12</v>
@@ -1975,12 +1915,12 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="47" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="48" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B12">
         <v>10</v>
@@ -1994,7 +1934,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="49" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B13">
         <v>10</v>
@@ -2045,7 +1985,7 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2054,7 +1994,7 @@
         <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E2" t="s">
         <v>18</v>
@@ -2063,15 +2003,15 @@
         <v>168</v>
       </c>
       <c r="G2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H2" t="s">
         <v>180</v>
-      </c>
-      <c r="H2" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B3">
         <v>5</v>
@@ -2080,7 +2020,7 @@
         <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E3" t="s">
         <v>19</v>
@@ -2089,15 +2029,15 @@
         <v>168</v>
       </c>
       <c r="G3" t="s">
+        <v>179</v>
+      </c>
+      <c r="H3" t="s">
         <v>180</v>
-      </c>
-      <c r="H3" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B4">
         <v>9</v>
@@ -2106,7 +2046,7 @@
         <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E4" t="s">
         <v>18</v>
@@ -2115,15 +2055,15 @@
         <v>168</v>
       </c>
       <c r="G4" t="s">
+        <v>179</v>
+      </c>
+      <c r="H4" t="s">
         <v>180</v>
-      </c>
-      <c r="H4" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B5">
         <v>13</v>
@@ -2132,7 +2072,7 @@
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E5" t="s">
         <v>19</v>
@@ -2141,24 +2081,24 @@
         <v>168</v>
       </c>
       <c r="G5" t="s">
+        <v>179</v>
+      </c>
+      <c r="H5" t="s">
         <v>180</v>
-      </c>
-      <c r="H5" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E6" t="s">
         <v>18</v>
@@ -2167,24 +2107,24 @@
         <v>168</v>
       </c>
       <c r="G6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H6" t="s">
         <v>180</v>
-      </c>
-      <c r="H6" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E7" t="s">
         <v>19</v>
@@ -2193,24 +2133,24 @@
         <v>168</v>
       </c>
       <c r="G7" t="s">
+        <v>179</v>
+      </c>
+      <c r="H7" t="s">
         <v>180</v>
-      </c>
-      <c r="H7" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B8">
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E8" t="s">
         <v>18</v>
@@ -2219,24 +2159,24 @@
         <v>168</v>
       </c>
       <c r="G8" t="s">
+        <v>179</v>
+      </c>
+      <c r="H8" t="s">
         <v>180</v>
-      </c>
-      <c r="H8" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B9">
         <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E9" t="s">
         <v>19</v>
@@ -2245,15 +2185,15 @@
         <v>168</v>
       </c>
       <c r="G9" t="s">
+        <v>179</v>
+      </c>
+      <c r="H9" t="s">
         <v>180</v>
-      </c>
-      <c r="H9" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B10">
         <v>3</v>
@@ -2262,7 +2202,7 @@
         <v>21</v>
       </c>
       <c r="D10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E10" t="s">
         <v>18</v>
@@ -2271,15 +2211,15 @@
         <v>168</v>
       </c>
       <c r="G10" t="s">
+        <v>179</v>
+      </c>
+      <c r="H10" t="s">
         <v>180</v>
-      </c>
-      <c r="H10" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B11">
         <v>7</v>
@@ -2288,7 +2228,7 @@
         <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E11" t="s">
         <v>19</v>
@@ -2297,15 +2237,15 @@
         <v>168</v>
       </c>
       <c r="G11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H11" t="s">
         <v>180</v>
-      </c>
-      <c r="H11" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -2314,7 +2254,7 @@
         <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E12" t="s">
         <v>18</v>
@@ -2323,15 +2263,15 @@
         <v>168</v>
       </c>
       <c r="G12" t="s">
+        <v>179</v>
+      </c>
+      <c r="H12" t="s">
         <v>180</v>
-      </c>
-      <c r="H12" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B13">
         <v>15</v>
@@ -2340,7 +2280,7 @@
         <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E13" t="s">
         <v>19</v>
@@ -2349,24 +2289,24 @@
         <v>168</v>
       </c>
       <c r="G13" t="s">
+        <v>179</v>
+      </c>
+      <c r="H13" t="s">
         <v>180</v>
-      </c>
-      <c r="H13" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B14">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E14" t="s">
         <v>18</v>
@@ -2375,24 +2315,24 @@
         <v>168</v>
       </c>
       <c r="G14" t="s">
+        <v>179</v>
+      </c>
+      <c r="H14" t="s">
         <v>180</v>
-      </c>
-      <c r="H14" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B15">
         <v>8</v>
       </c>
       <c r="C15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E15" t="s">
         <v>19</v>
@@ -2401,24 +2341,24 @@
         <v>168</v>
       </c>
       <c r="G15" t="s">
+        <v>179</v>
+      </c>
+      <c r="H15" t="s">
         <v>180</v>
-      </c>
-      <c r="H15" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B16">
         <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E16" t="s">
         <v>18</v>
@@ -2427,24 +2367,24 @@
         <v>168</v>
       </c>
       <c r="G16" t="s">
+        <v>179</v>
+      </c>
+      <c r="H16" t="s">
         <v>180</v>
-      </c>
-      <c r="H16" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B17">
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D17" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E17" t="s">
         <v>19</v>
@@ -2453,10 +2393,10 @@
         <v>168</v>
       </c>
       <c r="G17" t="s">
+        <v>179</v>
+      </c>
+      <c r="H17" t="s">
         <v>180</v>
-      </c>
-      <c r="H17" t="s">
-        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2469,14 +2409,14 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.90625" customWidth="1"/>
-    <col min="2" max="2" width="23.36328125" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" customWidth="1"/>
-    <col min="4" max="4" width="21.6328125" customWidth="1"/>
-    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="1" max="1" width="39.88671875" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21">
+    <row r="1" spans="1:6" ht="20.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2536,7 +2476,7 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:6" ht="31.2">
+    <row r="9" spans="1:6" ht="31.5">
       <c r="A9" s="4" t="s">
         <v>1</v>
       </c>
@@ -2544,7 +2484,7 @@
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:6" ht="46.8">
+    <row r="10" spans="1:6" ht="47.25">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
@@ -2644,7 +2584,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.6">
+    <row r="15" spans="1:6" ht="15.75">
       <c r="A15" s="9" t="s">
         <v>9</v>
       </c>
@@ -2665,7 +2605,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.6">
+    <row r="16" spans="1:6" ht="15.75">
       <c r="A16" s="9"/>
       <c r="B16" s="11" t="s">
         <v>11</v>
@@ -2688,11 +2628,11 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" customWidth="1"/>
-    <col min="6" max="7" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" customWidth="1"/>
+    <col min="6" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21">
+    <row r="1" spans="1:7" ht="20.25">
       <c r="A1" s="12" t="s">
         <v>151</v>
       </c>
@@ -2735,7 +2675,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.6">
+    <row r="7" spans="1:7" ht="15.75">
       <c r="A7" s="13" t="s">
         <v>149</v>
       </c>
@@ -2885,14 +2825,14 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="12.6328125" customWidth="1"/>
-    <col min="3" max="3" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="12.08984375" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" customWidth="1"/>
+    <col min="7" max="7" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21">
+    <row r="1" spans="1:8" ht="20.25">
       <c r="A1" s="12" t="s">
         <v>35</v>
       </c>
@@ -2922,7 +2862,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.6">
+    <row r="8" spans="1:8" ht="15.75">
       <c r="B8" s="24" t="s">
         <v>36</v>
       </c>
@@ -2958,9 +2898,9 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.6">
+    <row r="11" spans="1:8" ht="15.75">
       <c r="B11" s="20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C11" s="21">
         <v>200</v>
@@ -2975,12 +2915,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.6">
+    <row r="12" spans="1:8" ht="15.75">
       <c r="F12" s="24" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15.6">
+    <row r="16" spans="1:8" ht="15.75">
       <c r="B16" s="24" t="s">
         <v>38</v>
       </c>
@@ -2993,7 +2933,7 @@
         <v>40</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" spans="2:4">
@@ -3029,14 +2969,14 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" customWidth="1"/>
-    <col min="4" max="4" width="13.6328125" customWidth="1"/>
+    <col min="2" max="2" width="11.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
     <col min="5" max="5" width="4" customWidth="1"/>
-    <col min="6" max="6" width="14.90625" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21">
+    <row r="1" spans="1:7" ht="20.25">
       <c r="A1" s="2" t="s">
         <v>155</v>
       </c>
@@ -3085,7 +3025,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.6">
+    <row r="9" spans="1:7" ht="15.75">
       <c r="A9" s="31" t="s">
         <v>56</v>
       </c>
@@ -3101,7 +3041,7 @@
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="1:7" ht="15.6">
+    <row r="10" spans="1:7" ht="15.75">
       <c r="A10" s="5"/>
       <c r="B10" s="28" t="s">
         <v>49</v>
@@ -3243,15 +3183,15 @@
   <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="29.6328125" customWidth="1"/>
-    <col min="2" max="2" width="27.6328125" customWidth="1"/>
-    <col min="3" max="3" width="25.08984375" customWidth="1"/>
-    <col min="4" max="4" width="23.81640625" customWidth="1"/>
-    <col min="5" max="5" width="22.36328125" customWidth="1"/>
-    <col min="6" max="6" width="25.54296875" customWidth="1"/>
+    <col min="1" max="1" width="29.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.109375" customWidth="1"/>
+    <col min="4" max="4" width="23.77734375" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" customWidth="1"/>
+    <col min="6" max="6" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17.399999999999999">
+    <row r="1" spans="1:14" ht="18">
       <c r="A1" s="34" t="s">
         <v>107</v>
       </c>
@@ -3268,7 +3208,7 @@
       <c r="L1" s="32"/>
       <c r="M1" s="32"/>
     </row>
-    <row r="2" spans="1:14" ht="15.6">
+    <row r="2" spans="1:14" ht="15.75">
       <c r="A2" s="35" t="s">
         <v>59</v>
       </c>
@@ -3285,7 +3225,7 @@
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
     </row>
-    <row r="3" spans="1:14" ht="15.6">
+    <row r="3" spans="1:14" ht="15.75">
       <c r="A3" s="35" t="s">
         <v>60</v>
       </c>
@@ -3302,7 +3242,7 @@
       <c r="L3" s="32"/>
       <c r="M3" s="32"/>
     </row>
-    <row r="4" spans="1:14" ht="15.6">
+    <row r="4" spans="1:14" ht="15.75">
       <c r="A4" t="s">
         <v>114</v>
       </c>
@@ -3313,7 +3253,7 @@
       <c r="L4" s="32"/>
       <c r="M4" s="32"/>
     </row>
-    <row r="5" spans="1:14" s="24" customFormat="1" ht="31.2">
+    <row r="5" spans="1:14" s="24" customFormat="1" ht="31.5">
       <c r="A5" s="24" t="s">
         <v>10</v>
       </c>
@@ -3454,10 +3394,10 @@
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.1796875" customWidth="1"/>
+    <col min="1" max="1" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17.399999999999999">
+    <row r="1" spans="1:3" ht="18">
       <c r="A1" s="34" t="s">
         <v>70</v>
       </c>
@@ -3467,12 +3407,12 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="20.399999999999999" customHeight="1">
+    <row r="3" spans="1:3" ht="20.45" customHeight="1">
       <c r="A3" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="19.8" thickBot="1">
+    <row r="5" spans="1:3" ht="20.25" thickBot="1">
       <c r="A5" s="42" t="s">
         <v>156</v>
       </c>
@@ -3485,7 +3425,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.6">
+    <row r="7" spans="1:3" ht="15.75">
       <c r="A7" s="24" t="s">
         <v>10</v>
       </c>
@@ -3534,7 +3474,7 @@
       </c>
       <c r="C12" s="39"/>
     </row>
-    <row r="13" spans="1:3" ht="15.6">
+    <row r="13" spans="1:3" ht="15.75">
       <c r="A13" s="24" t="s">
         <v>10</v>
       </c>
@@ -3572,12 +3512,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="19.8" thickBot="1">
+    <row r="18" spans="1:3" ht="20.25" thickBot="1">
       <c r="A18" s="42" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="16.2" thickTop="1">
+    <row r="19" spans="1:3" ht="16.5" thickTop="1">
       <c r="B19" s="24" t="s">
         <v>159</v>
       </c>
@@ -3606,12 +3546,12 @@
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="19.54296875" customWidth="1"/>
+    <col min="3" max="3" width="19.5546875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="11" max="11" width="11.453125" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.399999999999999">
+    <row r="1" spans="1:6" ht="18">
       <c r="A1" s="34" t="s">
         <v>82</v>
       </c>

</xml_diff>